<commit_message>
Add videographer and split media budgets across 4 roles
Keep daily total at USD 2,200 and monthly package at USD 44,000,
redistributed equally among cameraman, photographer, videographer
and community manager.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-cobertura-1-dia.xlsx
+++ b/docs/presupuesto-cobertura-1-dia.xlsx
@@ -575,7 +575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D23"/>
+  <dimension ref="B2:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -594,14 +594,14 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Camarógrafo + Fotógrafo + Community Manager</t>
+          <t>Camarógrafo + Fotógrafo + Videógrafo + Community Manager</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Jornada de un día · honorarios distribuidos entre los tres perfiles</t>
+          <t>Jornada de un día · honorarios a partes iguales entre 4 perfiles</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>800</v>
+        <v>550</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -658,7 +658,7 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>700</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -667,66 +667,74 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
+          <t>VIDEÓGRAFO (1 día)</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="12" ht="26" customHeight="1">
+      <c r="B12" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="9" t="inlineStr">
+        <is>
           <t>COMMUNITY MANAGER (1 día)</t>
         </is>
       </c>
-      <c r="D11" s="10" t="n">
-        <v>700</v>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="B13" s="11" t="inlineStr">
+      <c r="D12" s="10" t="n">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>TOTAL 1 DÍA</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n"/>
-      <c r="D13" s="12">
-        <f>SUM(D9:D11)</f>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="12">
+        <f>SUM(D9:D12)</f>
         <v/>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="13" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>RESUMEN</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n"/>
-      <c r="D15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="15" t="inlineStr">
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t>Inversión total</t>
         </is>
       </c>
-      <c r="C16" s="5" t="n"/>
-      <c r="D16" s="16">
-        <f>D13</f>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="16">
+        <f>D14</f>
         <v/>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="17" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>Condiciones</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="18" t="inlineStr">
-        <is>
-          <t>• Incluye camarógrafo, fotógrafo y community manager según detalle.
+    <row r="20">
+      <c r="B20" s="18" t="inlineStr">
+        <is>
+          <t>• Incluye camarógrafo, fotógrafo, videógrafo y community manager.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Total: USD 2,200.</t>
         </is>
       </c>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="19" t="n"/>
       <c r="C20" s="19" t="n"/>
       <c r="D20" s="19" t="n"/>
     </row>
@@ -735,8 +743,13 @@
       <c r="C21" s="19" t="n"/>
       <c r="D21" s="19" t="n"/>
     </row>
-    <row r="23">
-      <c r="B23" s="20" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="19" t="n"/>
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="20" t="inlineStr">
         <is>
           <t>TOTAL 1 DÍA · Presupuesto cliente · 1 hoja</t>
         </is>
@@ -744,13 +757,13 @@
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="B13:C13"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B19:D21"/>
     <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B20:D22"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Prioritize media role rates instead of equal split
Keep USD 2,200/day and USD 44,000/month totals, with differentiated
amounts: videographer, cameraman, photographer, then community manager.

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-cobertura-1-dia.xlsx
+++ b/docs/presupuesto-cobertura-1-dia.xlsx
@@ -594,14 +594,14 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Camarógrafo + Fotógrafo + Videógrafo + Community Manager</t>
+          <t>Videógrafo + Camarógrafo + Fotógrafo + Community Manager</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Jornada de un día · honorarios a partes iguales entre 4 perfiles</t>
+          <t>Jornada de un día · montos priorizados por cargo</t>
         </is>
       </c>
     </row>
@@ -641,11 +641,11 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>CAMARÓGRAFO (1 día)</t>
+          <t>VIDEÓGRAFO (1 día)</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>550</v>
+        <v>700</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
@@ -654,11 +654,11 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>FOTÓGRAFO (1 día)</t>
+          <t>CAMARÓGRAFO (1 día)</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>550</v>
+        <v>600</v>
       </c>
     </row>
     <row r="11" ht="26" customHeight="1">
@@ -667,11 +667,11 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>VIDEÓGRAFO (1 día)</t>
+          <t>FOTÓGRAFO (1 día)</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>550</v>
+        <v>500</v>
       </c>
     </row>
     <row r="12" ht="26" customHeight="1">
@@ -684,7 +684,7 @@
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>550</v>
+        <v>400</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
@@ -730,7 +730,7 @@
     <row r="20">
       <c r="B20" s="18" t="inlineStr">
         <is>
-          <t>• Incluye camarógrafo, fotógrafo, videógrafo y community manager.
+          <t>• Incluye videógrafo, camarógrafo, fotógrafo y community manager.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Total: USD 2,200.</t>
         </is>

</xml_diff>

<commit_message>
Publish v2 media budgets with prioritized role amounts
Add cache-busting v2 filenames and an explicit distribution line so
clients download the unequal rates ($700/$600/$500/$400 daily).

Co-authored-by: crios82-max <crios82-max@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/presupuesto-cobertura-1-dia.xlsx
+++ b/docs/presupuesto-cobertura-1-dia.xlsx
@@ -95,13 +95,13 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00111A2D"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00111A2D"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <i val="1"/>
-      <color rgb="0094A3B8"/>
-      <sz val="8"/>
     </font>
   </fonts>
   <fills count="8">
@@ -168,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -187,7 +187,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -204,12 +204,15 @@
     <xf numFmtId="164" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -601,7 +604,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Jornada de un día · montos priorizados por cargo</t>
+          <t>Jornada de un día · montos PRIORIZADOS (no iguales)</t>
         </is>
       </c>
     </row>
@@ -694,9 +697,8 @@
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
-      <c r="D14" s="12">
-        <f>SUM(D9:D12)</f>
-        <v/>
+      <c r="D14" s="12" t="n">
+        <v>2200</v>
       </c>
     </row>
     <row r="16">
@@ -715,54 +717,56 @@
         </is>
       </c>
       <c r="C17" s="5" t="n"/>
-      <c r="D17" s="16">
-        <f>D14</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
+      <c r="D17" s="16" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
       <c r="B19" s="17" t="inlineStr">
         <is>
+          <t>Distribución: VIDEÓGRAFO $700 · CAMARÓGRAFO $600 · FOTÓGRAFO $500 · COMMUNITY MANAGER $400</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="n"/>
+      <c r="D19" s="18" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="19" t="inlineStr">
+        <is>
           <t>Condiciones</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>• Incluye videógrafo, camarógrafo, fotógrafo y community manager.
+    <row r="22">
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t>• Montos distintos por cargo (priorizados). No son iguales.
 • Validez del presupuesto: 15 días. Montos en dólares estadounidenses (USD).
 • Total: USD 2,200.</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
+      <c r="C22" s="21" t="n"/>
+      <c r="D22" s="21" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="21" t="n"/>
+      <c r="D23" s="21" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="20" t="inlineStr">
-        <is>
-          <t>TOTAL 1 DÍA · Presupuesto cliente · 1 hoja</t>
-        </is>
-      </c>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="21" t="n"/>
+      <c r="D24" s="21" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="B3:D3"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B22:D24"/>
     <mergeCell ref="B4:D4"/>
     <mergeCell ref="B16:D16"/>
     <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B20:D22"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B2:D2"/>
   </mergeCells>

</xml_diff>